<commit_message>
Code refactoring - Utterance KA
</commit_message>
<xml_diff>
--- a/Utterances/Annotations_Tests/Test1/Test1_consolidation.xlsx
+++ b/Utterances/Annotations_Tests/Test1/Test1_consolidation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10608"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katja/Dropbox/Doktorat/ParlaMint/Sentiment_annotation/Sentiment_aggregation/Annotations_Tests/Test1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katjameden/Library/CloudStorage/Dropbox/Projects/ParlaMint/Sentiment_annotation/ParlaMint_Sentiment/Utterances/Annotations_Tests/Test1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D90951AA-B27E-6A47-8AB9-B8903094BD0E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0431991-B29E-FB4A-ADA9-F522814C9593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="500" windowWidth="28040" windowHeight="16220" xr2:uid="{8874B2B3-69C9-AF40-98BC-CC3CD12E1CDB}"/>
+    <workbookView xWindow="380" yWindow="760" windowWidth="28040" windowHeight="16220" xr2:uid="{8874B2B3-69C9-AF40-98BC-CC3CD12E1CDB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -57,12 +57,6 @@
     <t>text</t>
   </si>
   <si>
-    <t>tamara_tag</t>
-  </si>
-  <si>
-    <t>katja_tag</t>
-  </si>
-  <si>
     <t>tamara_comments</t>
   </si>
   <si>
@@ -277,6 +271,12 @@
   </si>
   <si>
     <t>chair</t>
+  </si>
+  <si>
+    <t>tag_tamara</t>
+  </si>
+  <si>
+    <t>tag_katja</t>
   </si>
 </sst>
 </file>
@@ -655,498 +655,498 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
+        <v>73</v>
+      </c>
+      <c r="J1" t="s">
         <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>75</v>
-      </c>
-      <c r="J1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="J2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="85" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="G3" t="b">
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="119" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="F4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="J4" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="136" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="F5" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>27</v>
-      </c>
       <c r="H5" t="b">
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="F6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="I6" t="b">
         <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="F7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D7" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="I7" t="b">
         <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="I8" t="b">
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:10" ht="272" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>39</v>
-      </c>
       <c r="J9" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:10" ht="221" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="E10" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C10" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="F10" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="E10" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="J10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="51" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>43</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E11" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="F11" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="C11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>48</v>
-      </c>
       <c r="H11" t="b">
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:10" ht="85" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="F12" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="C12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" t="s">
-        <v>42</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="F12" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="J12" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:10" ht="34" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" t="s">
+        <v>9</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="F13" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="C13" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13" s="1" t="s">
-        <v>56</v>
-      </c>
       <c r="I13" t="b">
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:10" ht="85" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="F14" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C14" t="s">
-        <v>16</v>
-      </c>
-      <c r="D14" t="s">
-        <v>16</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F14" s="1" t="s">
-        <v>60</v>
-      </c>
       <c r="J14" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="15" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D15" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I15" t="b">
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C16" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D16" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I16" t="b">
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C17" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D17" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C18" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D18" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I18" t="b">
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="17" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C19" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D19" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="I19" t="b">
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
     </row>
     <row r="20" spans="1:10" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C20" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B20" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C20" t="s">
-        <v>16</v>
-      </c>
-      <c r="D20" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="J20" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>